<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-05
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B246"/>
+  <dimension ref="A1:B247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37842,6 +37842,18 @@
       <c r="B246" s="39" t="inlineStr">
         <is>
           <t>02, 04, 06, 19, 24, 25, 29, 32, 33, 36, 37, 39, 41, 45, 46, 47, 53, 57, 63, 71</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-05  Sáb</t>
+        </is>
+      </c>
+      <c r="B247" s="39" t="inlineStr">
+        <is>
+          <t>01, 05, 08, 10, 18, 23, 24, 27, 33, 35, 39, 42, 43, 45, 47, 50, 54, 55, 69, 78</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-06
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B247"/>
+  <dimension ref="A1:B248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37854,6 +37854,18 @@
       <c r="B247" s="39" t="inlineStr">
         <is>
           <t>01, 05, 08, 10, 18, 23, 24, 27, 33, 35, 39, 42, 43, 45, 47, 50, 54, 55, 69, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-06  Dom</t>
+        </is>
+      </c>
+      <c r="B248" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 06, 10, 19, 20, 26, 37, 38, 42, 47, 52, 53, 55, 60, 64, 68, 69, 75, 79</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +0 Pool hasta 2026-09-08
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B248"/>
+  <dimension ref="A1:B249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37866,6 +37866,18 @@
       <c r="B248" s="39" t="inlineStr">
         <is>
           <t>01, 02, 06, 10, 19, 20, 26, 37, 38, 42, 47, 52, 53, 55, 60, 64, 68, 69, 75, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-08  Mar</t>
+        </is>
+      </c>
+      <c r="B249" s="39" t="inlineStr">
+        <is>
+          <t>03, 08, 26, 32, 33, 34, 41, 42, 43, 44, 45, 46, 55, 59, 64, 66, 71, 74, 77, 79</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-09
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B249"/>
+  <dimension ref="A1:B250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37878,6 +37878,18 @@
       <c r="B249" s="39" t="inlineStr">
         <is>
           <t>03, 08, 26, 32, 33, 34, 41, 42, 43, 44, 45, 46, 55, 59, 64, 66, 71, 74, 77, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-09  Mié</t>
+        </is>
+      </c>
+      <c r="B250" s="39" t="inlineStr">
+        <is>
+          <t>09, 10, 13, 16, 21, 25, 32, 38, 40, 46, 47, 49, 51, 53, 54, 58, 63, 74, 75, 77</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-10
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B250"/>
+  <dimension ref="A1:B251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37890,6 +37890,18 @@
       <c r="B250" s="39" t="inlineStr">
         <is>
           <t>09, 10, 13, 16, 21, 25, 32, 38, 40, 46, 47, 49, 51, 53, 54, 58, 63, 74, 75, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-10  Jue</t>
+        </is>
+      </c>
+      <c r="B251" s="39" t="inlineStr">
+        <is>
+          <t>02, 07, 10, 16, 21, 30, 31, 34, 36, 39, 40, 42, 43, 48, 56, 60, 63, 65, 69, 77</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-11
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B251"/>
+  <dimension ref="A1:B252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37902,6 +37902,18 @@
       <c r="B251" s="39" t="inlineStr">
         <is>
           <t>02, 07, 10, 16, 21, 30, 31, 34, 36, 39, 40, 42, 43, 48, 56, 60, 63, 65, 69, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-11  Vie</t>
+        </is>
+      </c>
+      <c r="B252" s="39" t="inlineStr">
+        <is>
+          <t>01, 04, 11, 13, 16, 17, 28, 39, 40, 43, 46, 50, 52, 54, 56, 57, 59, 60, 68, 73</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-12
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B252"/>
+  <dimension ref="A1:B253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37914,6 +37914,18 @@
       <c r="B252" s="39" t="inlineStr">
         <is>
           <t>01, 04, 11, 13, 16, 17, 28, 39, 40, 43, 46, 50, 52, 54, 56, 57, 59, 60, 68, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-12  Sáb</t>
+        </is>
+      </c>
+      <c r="B253" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 07, 09, 12, 17, 22, 29, 35, 36, 38, 40, 42, 45, 62, 69, 74, 76, 79, 80</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-13
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B253"/>
+  <dimension ref="A1:B254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37926,6 +37926,18 @@
       <c r="B253" s="39" t="inlineStr">
         <is>
           <t>01, 02, 07, 09, 12, 17, 22, 29, 35, 36, 38, 40, 42, 45, 62, 69, 74, 76, 79, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-13  Dom</t>
+        </is>
+      </c>
+      <c r="B254" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 09, 13, 23, 31, 34, 43, 44, 47, 50, 56, 60, 61, 66, 68, 70, 71, 74, 76</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-14
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B254"/>
+  <dimension ref="A1:B255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37938,6 +37938,18 @@
       <c r="B254" s="39" t="inlineStr">
         <is>
           <t>02, 04, 09, 13, 23, 31, 34, 43, 44, 47, 50, 56, 60, 61, 66, 68, 70, 71, 74, 76</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-14  Lun</t>
+        </is>
+      </c>
+      <c r="B255" s="39" t="inlineStr">
+        <is>
+          <t>02, 04, 14, 17, 26, 32, 40, 46, 48, 51, 53, 54, 55, 56, 57, 58, 59, 69, 74, 75</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-15
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B255"/>
+  <dimension ref="A1:B256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37950,6 +37950,18 @@
       <c r="B255" s="39" t="inlineStr">
         <is>
           <t>02, 04, 14, 17, 26, 32, 40, 46, 48, 51, 53, 54, 55, 56, 57, 58, 59, 69, 74, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-15  Mar</t>
+        </is>
+      </c>
+      <c r="B256" s="39" t="inlineStr">
+        <is>
+          <t>04, 07, 09, 12, 15, 17, 27, 29, 30, 34, 35, 36, 40, 43, 47, 50, 53, 56, 67, 75</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-16
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B256"/>
+  <dimension ref="A1:B257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37962,6 +37962,18 @@
       <c r="B256" s="39" t="inlineStr">
         <is>
           <t>04, 07, 09, 12, 15, 17, 27, 29, 30, 34, 35, 36, 40, 43, 47, 50, 53, 56, 67, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-16  Mié</t>
+        </is>
+      </c>
+      <c r="B257" s="39" t="inlineStr">
+        <is>
+          <t>05, 11, 13, 16, 21, 27, 29, 32, 33, 42, 43, 47, 50, 53, 55, 59, 60, 68, 69, 74</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-17
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B257"/>
+  <dimension ref="A1:B258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37974,6 +37974,18 @@
       <c r="B257" s="39" t="inlineStr">
         <is>
           <t>05, 11, 13, 16, 21, 27, 29, 32, 33, 42, 43, 47, 50, 53, 55, 59, 60, 68, 69, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-17  Jue</t>
+        </is>
+      </c>
+      <c r="B258" s="39" t="inlineStr">
+        <is>
+          <t>12, 17, 19, 22, 23, 30, 34, 38, 40, 45, 46, 49, 50, 54, 55, 58, 59, 67, 72, 74</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-18
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B258"/>
+  <dimension ref="A1:B259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37986,6 +37986,18 @@
       <c r="B258" s="39" t="inlineStr">
         <is>
           <t>12, 17, 19, 22, 23, 30, 34, 38, 40, 45, 46, 49, 50, 54, 55, 58, 59, 67, 72, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-18  Vie</t>
+        </is>
+      </c>
+      <c r="B259" s="39" t="inlineStr">
+        <is>
+          <t>03, 04, 06, 11, 12, 14, 18, 20, 21, 22, 24, 32, 35, 37, 41, 42, 55, 56, 64, 74</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-19
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B259"/>
+  <dimension ref="A1:B260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37998,6 +37998,18 @@
       <c r="B259" s="39" t="inlineStr">
         <is>
           <t>03, 04, 06, 11, 12, 14, 18, 20, 21, 22, 24, 32, 35, 37, 41, 42, 55, 56, 64, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-19  Sáb</t>
+        </is>
+      </c>
+      <c r="B260" s="39" t="inlineStr">
+        <is>
+          <t>02, 09, 14, 15, 17, 19, 21, 28, 30, 31, 34, 37, 41, 45, 49, 58, 60, 61, 71, 72</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-20
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B260"/>
+  <dimension ref="A1:B261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38010,6 +38010,18 @@
       <c r="B260" s="39" t="inlineStr">
         <is>
           <t>02, 09, 14, 15, 17, 19, 21, 28, 30, 31, 34, 37, 41, 45, 49, 58, 60, 61, 71, 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-20  Dom</t>
+        </is>
+      </c>
+      <c r="B261" s="39" t="inlineStr">
+        <is>
+          <t>01, 10, 12, 13, 17, 20, 24, 27, 29, 38, 46, 54, 55, 56, 62, 63, 65, 69, 78, 79</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-21
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B261"/>
+  <dimension ref="A1:B262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38022,6 +38022,18 @@
       <c r="B261" s="39" t="inlineStr">
         <is>
           <t>01, 10, 12, 13, 17, 20, 24, 27, 29, 38, 46, 54, 55, 56, 62, 63, 65, 69, 78, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-21  Lun</t>
+        </is>
+      </c>
+      <c r="B262" s="39" t="inlineStr">
+        <is>
+          <t>03, 07, 11, 16, 17, 18, 21, 22, 23, 24, 31, 33, 35, 36, 41, 43, 46, 49, 63, 64</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-22
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B262"/>
+  <dimension ref="A1:B263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38034,6 +38034,18 @@
       <c r="B262" s="39" t="inlineStr">
         <is>
           <t>03, 07, 11, 16, 17, 18, 21, 22, 23, 24, 31, 33, 35, 36, 41, 43, 46, 49, 63, 64</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-22  Mar</t>
+        </is>
+      </c>
+      <c r="B263" s="39" t="inlineStr">
+        <is>
+          <t>05, 12, 16, 19, 22, 27, 29, 33, 40, 44, 45, 47, 48, 49, 59, 61, 64, 68, 69, 74</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-23
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B263"/>
+  <dimension ref="A1:B264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38046,6 +38046,18 @@
       <c r="B263" s="39" t="inlineStr">
         <is>
           <t>05, 12, 16, 19, 22, 27, 29, 33, 40, 44, 45, 47, 48, 49, 59, 61, 64, 68, 69, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-23  Mié</t>
+        </is>
+      </c>
+      <c r="B264" s="39" t="inlineStr">
+        <is>
+          <t>01, 04, 12, 19, 23, 28, 29, 36, 43, 45, 46, 49, 53, 58, 62, 63, 65, 66, 67, 71</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-24
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B264"/>
+  <dimension ref="A1:B265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38058,6 +38058,18 @@
       <c r="B264" s="39" t="inlineStr">
         <is>
           <t>01, 04, 12, 19, 23, 28, 29, 36, 43, 45, 46, 49, 53, 58, 62, 63, 65, 66, 67, 71</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-24  Jue</t>
+        </is>
+      </c>
+      <c r="B265" s="39" t="inlineStr">
+        <is>
+          <t>03, 09, 12, 16, 19, 23, 24, 31, 37, 39, 43, 57, 59, 61, 64, 65, 69, 70, 74, 77</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-26
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B265"/>
+  <dimension ref="A1:B266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38070,6 +38070,18 @@
       <c r="B265" s="39" t="inlineStr">
         <is>
           <t>03, 09, 12, 16, 19, 23, 24, 31, 37, 39, 43, 57, 59, 61, 64, 65, 69, 70, 74, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-26  Sáb</t>
+        </is>
+      </c>
+      <c r="B266" s="39" t="inlineStr">
+        <is>
+          <t>04, 07, 09, 11, 13, 21, 22, 23, 26, 31, 32, 36, 47, 54, 58, 61, 64, 69, 71, 75</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-27
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B266"/>
+  <dimension ref="A1:B267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38082,6 +38082,18 @@
       <c r="B266" s="39" t="inlineStr">
         <is>
           <t>04, 07, 09, 11, 13, 21, 22, 23, 26, 31, 32, 36, 47, 54, 58, 61, 64, 69, 71, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-27  Dom</t>
+        </is>
+      </c>
+      <c r="B267" s="39" t="inlineStr">
+        <is>
+          <t>05, 15, 18, 19, 27, 29, 31, 33, 41, 42, 43, 46, 47, 55, 57, 58, 59, 62, 71, 80</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-28
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B267"/>
+  <dimension ref="A1:B268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38094,6 +38094,18 @@
       <c r="B267" s="39" t="inlineStr">
         <is>
           <t>05, 15, 18, 19, 27, 29, 31, 33, 41, 42, 43, 46, 47, 55, 57, 58, 59, 62, 71, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-28  Lun</t>
+        </is>
+      </c>
+      <c r="B268" s="39" t="inlineStr">
+        <is>
+          <t>02, 15, 16, 17, 18, 22, 24, 25, 27, 28, 41, 43, 46, 56, 59, 63, 64, 68, 70, 75</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-09-29
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B268"/>
+  <dimension ref="A1:B269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38106,6 +38106,18 @@
       <c r="B268" s="39" t="inlineStr">
         <is>
           <t>02, 15, 16, 17, 18, 22, 24, 25, 27, 28, 41, 43, 46, 56, 59, 63, 64, 68, 70, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-29  Mar</t>
+        </is>
+      </c>
+      <c r="B269" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 14, 20, 22, 25, 28, 29, 36, 38, 41, 49, 51, 54, 55, 58, 61, 64, 76, 77</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +2 Kino, +2 Pool hasta 2026-10-01
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B269"/>
+  <dimension ref="A1:B271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38118,6 +38118,30 @@
       <c r="B269" s="39" t="inlineStr">
         <is>
           <t>02, 03, 14, 20, 22, 25, 28, 29, 36, 38, 41, 49, 51, 54, 55, 58, 61, 64, 76, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="39" t="inlineStr">
+        <is>
+          <t>2026-09-30  Mié</t>
+        </is>
+      </c>
+      <c r="B270" s="39" t="inlineStr">
+        <is>
+          <t>03, 05, 12, 13, 14, 19, 20, 24, 30, 31, 38, 43, 46, 51, 59, 60, 62, 64, 65, 69</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-01  Jue</t>
+        </is>
+      </c>
+      <c r="B271" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 04, 05, 15, 22, 42, 45, 47, 49, 54, 55, 58, 60, 66, 67, 72, 74, 75, 79</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-02
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B271"/>
+  <dimension ref="A1:B272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38142,6 +38142,18 @@
       <c r="B271" s="39" t="inlineStr">
         <is>
           <t>01, 02, 04, 05, 15, 22, 42, 45, 47, 49, 54, 55, 58, 60, 66, 67, 72, 74, 75, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-02  Vie</t>
+        </is>
+      </c>
+      <c r="B272" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 05, 09, 19, 22, 24, 26, 37, 39, 40, 42, 49, 51, 55, 57, 60, 68, 71, 73</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-04
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B272"/>
+  <dimension ref="A1:B273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38154,6 +38154,18 @@
       <c r="B272" s="39" t="inlineStr">
         <is>
           <t>02, 03, 05, 09, 19, 22, 24, 26, 37, 39, 40, 42, 49, 51, 55, 57, 60, 68, 71, 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-04  Dom</t>
+        </is>
+      </c>
+      <c r="B273" s="39" t="inlineStr">
+        <is>
+          <t>04, 07, 08, 09, 11, 19, 23, 32, 36, 38, 42, 46, 49, 51, 68, 69, 70, 71, 73, 74</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-05
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B273"/>
+  <dimension ref="A1:B274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38166,6 +38166,18 @@
       <c r="B273" s="39" t="inlineStr">
         <is>
           <t>04, 07, 08, 09, 11, 19, 23, 32, 36, 38, 42, 46, 49, 51, 68, 69, 70, 71, 73, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-05  Lun</t>
+        </is>
+      </c>
+      <c r="B274" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 05, 12, 14, 16, 21, 22, 24, 27, 37, 38, 39, 50, 51, 52, 61, 69, 71, 75</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-06
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B274"/>
+  <dimension ref="A1:B275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38178,6 +38178,18 @@
       <c r="B274" s="39" t="inlineStr">
         <is>
           <t>01, 02, 05, 12, 14, 16, 21, 22, 24, 27, 37, 38, 39, 50, 51, 52, 61, 69, 71, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-06  Mar</t>
+        </is>
+      </c>
+      <c r="B275" s="39" t="inlineStr">
+        <is>
+          <t>01, 02, 03, 06, 11, 13, 16, 17, 21, 27, 32, 40, 43, 46, 47, 51, 57, 66, 69, 78</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-07
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B275"/>
+  <dimension ref="A1:B276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38190,6 +38190,18 @@
       <c r="B275" s="39" t="inlineStr">
         <is>
           <t>01, 02, 03, 06, 11, 13, 16, 17, 21, 27, 32, 40, 43, 46, 47, 51, 57, 66, 69, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-07  Mié</t>
+        </is>
+      </c>
+      <c r="B276" s="39" t="inlineStr">
+        <is>
+          <t>01, 07, 10, 11, 12, 17, 24, 25, 29, 32, 35, 46, 48, 50, 54, 64, 65, 71, 79, 80</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-08
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B276"/>
+  <dimension ref="A1:B277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38202,6 +38202,18 @@
       <c r="B276" s="39" t="inlineStr">
         <is>
           <t>01, 07, 10, 11, 12, 17, 24, 25, 29, 32, 35, 46, 48, 50, 54, 64, 65, 71, 79, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-08  Jue</t>
+        </is>
+      </c>
+      <c r="B277" s="39" t="inlineStr">
+        <is>
+          <t>05, 06, 08, 14, 27, 28, 30, 35, 39, 41, 44, 46, 60, 63, 64, 65, 69, 73, 75, 77</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-09
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B277"/>
+  <dimension ref="A1:B278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38214,6 +38214,18 @@
       <c r="B277" s="39" t="inlineStr">
         <is>
           <t>05, 06, 08, 14, 27, 28, 30, 35, 39, 41, 44, 46, 60, 63, 64, 65, 69, 73, 75, 77</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-09  Vie</t>
+        </is>
+      </c>
+      <c r="B278" s="39" t="inlineStr">
+        <is>
+          <t>04, 06, 07, 09, 15, 23, 27, 30, 31, 32, 33, 45, 46, 52, 59, 68, 71, 72, 74, 79</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-12
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B278"/>
+  <dimension ref="A1:B279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38226,6 +38226,18 @@
       <c r="B278" s="39" t="inlineStr">
         <is>
           <t>04, 06, 07, 09, 15, 23, 27, 30, 31, 32, 33, 45, 46, 52, 59, 68, 71, 72, 74, 79</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-12  Lun</t>
+        </is>
+      </c>
+      <c r="B279" s="39" t="inlineStr">
+        <is>
+          <t>04, 07, 09, 12, 17, 19, 20, 24, 34, 36, 41, 48, 49, 52, 53, 56, 72, 73, 74, 78</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-13
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B279"/>
+  <dimension ref="A1:B280"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38238,6 +38238,18 @@
       <c r="B279" s="39" t="inlineStr">
         <is>
           <t>04, 07, 09, 12, 17, 19, 20, 24, 34, 36, 41, 48, 49, 52, 53, 56, 72, 73, 74, 78</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-13  Mar</t>
+        </is>
+      </c>
+      <c r="B280" s="39" t="inlineStr">
+        <is>
+          <t>02, 03, 04, 05, 10, 13, 20, 23, 27, 34, 37, 40, 44, 46, 47, 51, 59, 72, 74, 80</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-14
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B280"/>
+  <dimension ref="A1:B281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38250,6 +38250,18 @@
       <c r="B280" s="39" t="inlineStr">
         <is>
           <t>02, 03, 04, 05, 10, 13, 20, 23, 27, 34, 37, 40, 44, 46, 47, 51, 59, 72, 74, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-14  Mié</t>
+        </is>
+      </c>
+      <c r="B281" s="39" t="inlineStr">
+        <is>
+          <t>03, 06, 07, 13, 14, 21, 28, 31, 36, 42, 46, 51, 52, 63, 68, 70, 72, 76, 78, 80</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-15
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B281"/>
+  <dimension ref="A1:B282"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38262,6 +38262,18 @@
       <c r="B281" s="39" t="inlineStr">
         <is>
           <t>03, 06, 07, 13, 14, 21, 28, 31, 36, 42, 46, 51, 52, 63, 68, 70, 72, 76, 78, 80</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-15  Jue</t>
+        </is>
+      </c>
+      <c r="B282" s="39" t="inlineStr">
+        <is>
+          <t>02, 07, 11, 15, 16, 24, 32, 33, 35, 40, 42, 44, 45, 46, 51, 60, 65, 69, 71, 75</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-16
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B282"/>
+  <dimension ref="A1:B283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38274,6 +38274,18 @@
       <c r="B282" s="39" t="inlineStr">
         <is>
           <t>02, 07, 11, 15, 16, 24, 32, 33, 35, 40, 42, 44, 45, 46, 51, 60, 65, 69, 71, 75</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-16  Vie</t>
+        </is>
+      </c>
+      <c r="B283" s="39" t="inlineStr">
+        <is>
+          <t>06, 07, 10, 16, 17, 33, 40, 41, 43, 44, 46, 49, 50, 51, 55, 64, 65, 69, 73, 74</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
datos: +1 Kino, +1 Pool hasta 2026-10-17
</commit_message>
<xml_diff>
--- a/data/kino_2010_a_hoy_COMPLETO.xlsx
+++ b/data/kino_2010_a_hoy_COMPLETO.xlsx
@@ -34896,7 +34896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B283"/>
+  <dimension ref="A1:B284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38286,6 +38286,18 @@
       <c r="B283" s="39" t="inlineStr">
         <is>
           <t>06, 07, 10, 16, 17, 33, 40, 41, 43, 44, 46, 49, 50, 51, 55, 64, 65, 69, 73, 74</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="39" t="inlineStr">
+        <is>
+          <t>2026-10-17  Sáb</t>
+        </is>
+      </c>
+      <c r="B284" s="39" t="inlineStr">
+        <is>
+          <t>03, 06, 11, 14, 15, 17, 18, 20, 25, 26, 31, 34, 35, 36, 40, 41, 47, 49, 63, 72</t>
         </is>
       </c>
     </row>

</xml_diff>